<commit_message>
feat(register): import a filled register template from XLSX or CSV
Teams that fill the register template in Excel had to retype every row.
"Import a filled register" in the Save or restore menu reads the first
sheet in the browser. It matches columns by the field names in row 1,
skips the template's label row, and accepts option ids or visible English
or Arabic labels. Anything unrecognised is left blank and counted, never
guessed. Tiers are always recomputed from the answers, and rows without a
name or owner are skipped and counted.

The register template gains product and deployment columns. A unit test
imports the kit's own EN and AR templates, in both formats, and checks
their stated tiers. See ADR 012.
</commit_message>
<xml_diff>
--- a/public/templates/ar/register.xlsx
+++ b/public/templates/ar/register.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:T4"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -438,39 +438,45 @@
         <v>status</v>
       </c>
       <c r="G1" t="str">
+        <v>product</v>
+      </c>
+      <c r="H1" t="str">
+        <v>deployment</v>
+      </c>
+      <c r="I1" t="str">
         <v>runtime_ai</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>ai_type</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>impact</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>data</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>affected</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>autonomy</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>oversight</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>access</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>reversibility</v>
       </c>
-      <c r="P1" t="str">
+      <c r="R1" t="str">
         <v>tier</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>deep_dive_complete</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>updatedAt</v>
       </c>
     </row>
@@ -494,39 +500,45 @@
         <v>الحالة</v>
       </c>
       <c r="G2" t="str">
+        <v>المنتج</v>
+      </c>
+      <c r="H2" t="str">
+        <v>طريقة النشر</v>
+      </c>
+      <c r="I2" t="str">
         <v>هل يستخدم الحل الذكاء الاصطناعي أثناء تشغيله؟</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>نوع الذكاء الاصطناعي</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>على ماذا تؤثر مخرجات نظام الذكاء الاصطناعي؟</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>ما البيانات التي يستخدمها؟</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>من قد يتأثر؟</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>إلى أي مدى يعمل باستقلالية؟</v>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v>كيف يراجع البشر عمله؟</v>
       </c>
-      <c r="N2" t="str">
+      <c r="P2" t="str">
         <v>ما الذي يمكنه تغييره في الأنظمة الأخرى؟</v>
       </c>
-      <c r="O2" t="str">
+      <c r="Q2" t="str">
         <v>إذا أخطأ، هل يمكن التراجع عن النتيجة؟</v>
       </c>
-      <c r="P2" t="str">
+      <c r="R2" t="str">
         <v>مستوى المخاطر</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="S2" t="str">
         <v>التقييم المعمّق</v>
       </c>
-      <c r="R2" t="str">
+      <c r="T2" t="str">
         <v>آخر تحديث</v>
       </c>
     </row>
@@ -549,40 +561,40 @@
       <c r="F3" t="str">
         <v>production</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>yes</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>generative</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>public-info</v>
       </c>
-      <c r="J3" t="str">
+      <c r="L3" t="str">
         <v>none</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>public</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>monitored</v>
       </c>
-      <c r="M3" t="str">
+      <c r="O3" t="str">
         <v>exceptions</v>
       </c>
-      <c r="N3" t="str">
+      <c r="P3" t="str">
         <v>none</v>
       </c>
-      <c r="O3" t="str">
+      <c r="Q3" t="str">
         <v>easy</v>
       </c>
-      <c r="P3" t="str">
+      <c r="R3" t="str">
         <v>limited</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="S3" t="str">
         <v>false</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>2026-01-15</v>
       </c>
     </row>
@@ -605,46 +617,46 @@
       <c r="F4" t="str">
         <v>pilot</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>yes</v>
       </c>
-      <c r="H4" t="str">
+      <c r="J4" t="str">
         <v>agentic</v>
       </c>
-      <c r="I4" t="str">
+      <c r="K4" t="str">
         <v>recommend-individuals</v>
       </c>
-      <c r="J4" t="str">
+      <c r="L4" t="str">
         <v>personal</v>
       </c>
-      <c r="K4" t="str">
+      <c r="M4" t="str">
         <v>public</v>
       </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
         <v>monitored</v>
       </c>
-      <c r="M4" t="str">
+      <c r="O4" t="str">
         <v>exceptions</v>
       </c>
-      <c r="N4" t="str">
+      <c r="P4" t="str">
         <v>record</v>
       </c>
-      <c r="O4" t="str">
+      <c r="Q4" t="str">
         <v>easy</v>
       </c>
-      <c r="P4" t="str">
+      <c r="R4" t="str">
         <v>high</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="S4" t="str">
         <v>false</v>
       </c>
-      <c r="R4" t="str">
+      <c r="T4" t="str">
         <v>2026-01-15</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>